<commit_message>
Update project and PAYSYS data
</commit_message>
<xml_diff>
--- a/data/PAYSYS_Weekly_Project_Update_04-Sep-2026.xlsx
+++ b/data/PAYSYS_Weekly_Project_Update_04-Sep-2026.xlsx
@@ -115,9 +115,6 @@
     <t>UBPS Issue</t>
   </si>
   <si>
-    <t>Success response shared to channel but transactions failed at 1 Link end.</t>
-  </si>
-  <si>
     <t>RAAST Bulk Issue</t>
   </si>
   <si>
@@ -133,9 +130,6 @@
     <t>UAT awaited</t>
   </si>
   <si>
-    <t>Unable to connect please try again.</t>
-  </si>
-  <si>
     <t>Slot for UAT if Required.</t>
   </si>
   <si>
@@ -152,6 +146,12 @@
   </si>
   <si>
     <t>Debit Hold Failed at PAYSYS End</t>
+  </si>
+  <si>
+    <t>Session with PAYSYS on RAAST</t>
+  </si>
+  <si>
+    <t>Success response shared to channel but transactions failed at 1 Link end. Report Required of rejected trasnactions.</t>
   </si>
 </sst>
 </file>
@@ -597,7 +597,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -629,13 +629,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
@@ -645,13 +645,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
@@ -705,7 +705,7 @@
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -740,7 +740,7 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -759,7 +759,7 @@
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -778,7 +778,7 @@
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
@@ -794,7 +794,7 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
@@ -804,13 +804,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
@@ -829,7 +829,7 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>